<commit_message>
Fixed register start bits on rest of sheets. Removed note as it is no-longer relevant.
</commit_message>
<xml_diff>
--- a/To Add v2/Thermal - Pads.xlsx
+++ b/To Add v2/Thermal - Pads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5DD295-1DB1-4076-A817-8E87D5595FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF6F8C9-DA96-4028-A078-D27D055615AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="45">
   <si>
     <t>Totals</t>
   </si>
@@ -141,6 +141,36 @@
   </si>
   <si>
     <t> </t>
+  </si>
+  <si>
+    <t>5mmx5mm</t>
+  </si>
+  <si>
+    <t>https://www.arctic.de/media/3c/92/75/1664269110/Spec_Sheet_TP-3_EN.pdf</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Arctic</t>
+  </si>
+  <si>
+    <t>ACTPD00059A</t>
+  </si>
+  <si>
+    <t>Bulk Ordered</t>
+  </si>
+  <si>
+    <t>5mmx10mm</t>
+  </si>
+  <si>
+    <t>10mmx10mm</t>
+  </si>
+  <si>
+    <t>15mmx15mm</t>
   </si>
 </sst>
 </file>
@@ -205,7 +235,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -481,14 +519,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:X7"/>
+  <dimension ref="B1:X12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="35.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.26953125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.6328125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -510,43 +551,43 @@
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F2">
         <f t="shared" ref="F2:H2" si="1">COUNTA(F7:F9999)</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
@@ -554,7 +595,7 @@
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W2" t="s">
         <v>1</v>
@@ -570,7 +611,7 @@
       </c>
       <c r="X3">
         <f>MAX(C2:P2)</f>
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.35">
@@ -754,7 +795,187 @@
         <v>14</v>
       </c>
     </row>
+    <row r="8" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8">
+        <v>12</v>
+      </c>
+      <c r="H8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8" t="s">
+        <v>38</v>
+      </c>
+      <c r="M8" t="s">
+        <v>36</v>
+      </c>
+      <c r="N8" t="s">
+        <v>32</v>
+      </c>
+      <c r="P8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="E9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9">
+        <v>12</v>
+      </c>
+      <c r="H9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" t="s">
+        <v>40</v>
+      </c>
+      <c r="K9" t="s">
+        <v>37</v>
+      </c>
+      <c r="L9" t="s">
+        <v>38</v>
+      </c>
+      <c r="M9" t="s">
+        <v>36</v>
+      </c>
+      <c r="N9" t="s">
+        <v>32</v>
+      </c>
+      <c r="P9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="E10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10">
+        <v>13</v>
+      </c>
+      <c r="H10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" t="s">
+        <v>40</v>
+      </c>
+      <c r="K10" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" t="s">
+        <v>38</v>
+      </c>
+      <c r="M10" t="s">
+        <v>36</v>
+      </c>
+      <c r="N10" t="s">
+        <v>32</v>
+      </c>
+      <c r="P10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="E11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11">
+        <v>14</v>
+      </c>
+      <c r="H11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11" t="s">
+        <v>39</v>
+      </c>
+      <c r="J11" t="s">
+        <v>40</v>
+      </c>
+      <c r="K11" t="s">
+        <v>37</v>
+      </c>
+      <c r="L11" t="s">
+        <v>38</v>
+      </c>
+      <c r="M11" t="s">
+        <v>36</v>
+      </c>
+      <c r="N11" t="s">
+        <v>32</v>
+      </c>
+      <c r="P11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="E12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J12" t="s">
+        <v>40</v>
+      </c>
+      <c r="K12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M12" t="s">
+        <v>36</v>
+      </c>
+      <c r="N12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P12" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C7:P71">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(C7))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>